<commit_message>
Elv: graficos de partição finalizados
</commit_message>
<xml_diff>
--- a/res/tabela de partição.xlsx
+++ b/res/tabela de partição.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/480d9b848b88e342/MSS/_Zoo-Rebio/ZooRebio3-23_24/rebio23-part/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_B1E23327000965AC9047A4F15FFF14BAB25A30DE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF5A2312-69D2-467A-877B-D46D17667D89}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="6_{445A1B70-2E2A-4C5C-B9EA-91A8B12785EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21720" yWindow="-22425" windowWidth="21840" windowHeight="37920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,12 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
     <sheet name="tabela_final" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="144">
   <si>
     <t>Sistema</t>
   </si>
@@ -50,36 +50,9 @@
     <t>Seco</t>
   </si>
   <si>
-    <t>α1 (micro-habitat)</t>
-  </si>
-  <si>
-    <t>16.40%</t>
-  </si>
-  <si>
-    <t>21.17%</t>
-  </si>
-  <si>
-    <t>-12.27</t>
-  </si>
-  <si>
     <t>&lt; 0.001*</t>
   </si>
   <si>
-    <t>α2 (ponto)</t>
-  </si>
-  <si>
-    <t>28.84%</t>
-  </si>
-  <si>
-    <t>37.52%</t>
-  </si>
-  <si>
-    <t>-9.32</t>
-  </si>
-  <si>
-    <t>γ (Riqueza total)</t>
-  </si>
-  <si>
     <t>100.00%</t>
   </si>
   <si>
@@ -89,51 +62,9 @@
     <t>1.000</t>
   </si>
   <si>
-    <t>β1 (entre micro-habitats)</t>
-  </si>
-  <si>
-    <t>12.43%</t>
-  </si>
-  <si>
-    <t>16.35%</t>
-  </si>
-  <si>
-    <t>-4.84</t>
-  </si>
-  <si>
-    <t>β2 (entre pontos)</t>
-  </si>
-  <si>
-    <t>71.16%</t>
-  </si>
-  <si>
-    <t>62.48%</t>
-  </si>
-  <si>
-    <t>9.32</t>
-  </si>
-  <si>
     <t>Chuvoso</t>
   </si>
   <si>
-    <t>21.18%</t>
-  </si>
-  <si>
-    <t>-12.12</t>
-  </si>
-  <si>
-    <t>-9.29</t>
-  </si>
-  <si>
-    <t>16.33%</t>
-  </si>
-  <si>
-    <t>-4.70</t>
-  </si>
-  <si>
-    <t>9.29</t>
-  </si>
-  <si>
     <t>Riacho Barro Branco (BB)</t>
   </si>
   <si>
@@ -143,175 +74,385 @@
     <t>26.63%</t>
   </si>
   <si>
-    <t>-11.64</t>
-  </si>
-  <si>
     <t>35.04%</t>
   </si>
   <si>
-    <t>46.86%</t>
-  </si>
-  <si>
-    <t>-9.03</t>
-  </si>
-  <si>
     <t>14.81%</t>
   </si>
   <si>
-    <t>-4.66</t>
-  </si>
-  <si>
     <t>64.96%</t>
   </si>
   <si>
-    <t>53.14%</t>
-  </si>
-  <si>
-    <t>9.03</t>
-  </si>
-  <si>
-    <t>26.64%</t>
-  </si>
-  <si>
-    <t>-11.86</t>
+    <t>Partição Total (PT)</t>
+  </si>
+  <si>
+    <t>12.45%</t>
+  </si>
+  <si>
+    <t>19.42%</t>
+  </si>
+  <si>
+    <t>22.18%</t>
+  </si>
+  <si>
+    <t>73.28%</t>
+  </si>
+  <si>
+    <t>9.73%</t>
+  </si>
+  <si>
+    <t>51.09%</t>
+  </si>
+  <si>
+    <t>0.67</t>
+  </si>
+  <si>
+    <t>26.72%</t>
+  </si>
+  <si>
+    <t>23.72%</t>
+  </si>
+  <si>
+    <t>35.50%</t>
+  </si>
+  <si>
+    <t>83.75%</t>
+  </si>
+  <si>
+    <t>11.78%</t>
+  </si>
+  <si>
+    <t>48.25%</t>
+  </si>
+  <si>
+    <t>16.25%</t>
+  </si>
+  <si>
+    <t>Sistema</t>
+  </si>
+  <si>
+    <t>Período</t>
+  </si>
+  <si>
+    <t>Componente</t>
+  </si>
+  <si>
+    <t>Obs (%)</t>
+  </si>
+  <si>
+    <t>Esp (%)</t>
+  </si>
+  <si>
+    <t>SES</t>
+  </si>
+  <si>
+    <t>p-valor</t>
+  </si>
+  <si>
+    <t>Partição Total (PT)</t>
+  </si>
+  <si>
+    <t>Seco</t>
+  </si>
+  <si>
+    <t>12.45%</t>
+  </si>
+  <si>
+    <t>&lt; 0.001*</t>
+  </si>
+  <si>
+    <t>22.18%</t>
+  </si>
+  <si>
+    <t>73.28%</t>
+  </si>
+  <si>
+    <t>100.00%</t>
+  </si>
+  <si>
+    <t>0.00</t>
+  </si>
+  <si>
+    <t>1.000</t>
+  </si>
+  <si>
+    <t>9.73%</t>
+  </si>
+  <si>
+    <t>51.09%</t>
+  </si>
+  <si>
+    <t>26.72%</t>
+  </si>
+  <si>
+    <t>Chuvoso</t>
+  </si>
+  <si>
+    <t>23.72%</t>
+  </si>
+  <si>
+    <t>51.70%</t>
+  </si>
+  <si>
+    <t>35.50%</t>
+  </si>
+  <si>
+    <t>83.75%</t>
+  </si>
+  <si>
+    <t>11.78%</t>
+  </si>
+  <si>
+    <t>48.25%</t>
+  </si>
+  <si>
+    <t>16.25%</t>
+  </si>
+  <si>
+    <t>Riacho Barro Branco (BB)</t>
+  </si>
+  <si>
+    <t>20.23%</t>
+  </si>
+  <si>
+    <t>35.04%</t>
+  </si>
+  <si>
+    <t>14.81%</t>
+  </si>
+  <si>
+    <t>64.96%</t>
+  </si>
+  <si>
+    <t>24.24%</t>
+  </si>
+  <si>
+    <t>37.37%</t>
+  </si>
+  <si>
+    <t>13.13%</t>
+  </si>
+  <si>
+    <t>62.63%</t>
+  </si>
+  <si>
+    <t>Riacho Caiana (CA)</t>
+  </si>
+  <si>
+    <t>14.73%</t>
+  </si>
+  <si>
+    <t>22.47%</t>
+  </si>
+  <si>
+    <t>26.81%</t>
+  </si>
+  <si>
+    <t>12.08%</t>
+  </si>
+  <si>
+    <t>73.19%</t>
+  </si>
+  <si>
+    <t>30.83%</t>
+  </si>
+  <si>
+    <t>45.42%</t>
+  </si>
+  <si>
+    <t>14.60%</t>
+  </si>
+  <si>
+    <t>54.58%</t>
+  </si>
+  <si>
+    <t>α1 (Habitat)</t>
+  </si>
+  <si>
+    <t>19.42%</t>
+  </si>
+  <si>
+    <t>-21.96</t>
+  </si>
+  <si>
+    <t>α2 (Site)</t>
+  </si>
+  <si>
+    <t>34.43%</t>
+  </si>
+  <si>
+    <t>-17.38</t>
+  </si>
+  <si>
+    <t>α3 (Stream)</t>
+  </si>
+  <si>
+    <t>84.24%</t>
+  </si>
+  <si>
+    <t>-5.64</t>
+  </si>
+  <si>
+    <t>γ (Total richness)</t>
+  </si>
+  <si>
+    <t>β1 (Between habitats)</t>
+  </si>
+  <si>
+    <t>15.02%</t>
+  </si>
+  <si>
+    <t>-9.23</t>
+  </si>
+  <si>
+    <t>β2 (Between sites)</t>
+  </si>
+  <si>
+    <t>49.81%</t>
+  </si>
+  <si>
+    <t>0.67</t>
+  </si>
+  <si>
+    <t>0.535</t>
+  </si>
+  <si>
+    <t>β3 (Between streams)</t>
+  </si>
+  <si>
+    <t>15.76%</t>
+  </si>
+  <si>
+    <t>5.64</t>
+  </si>
+  <si>
+    <t>-46.09</t>
+  </si>
+  <si>
+    <t>69.42%</t>
+  </si>
+  <si>
+    <t>-36.07</t>
+  </si>
+  <si>
+    <t>96.40%</t>
+  </si>
+  <si>
+    <t>-9.73</t>
+  </si>
+  <si>
+    <t>17.72%</t>
+  </si>
+  <si>
+    <t>-7.60</t>
+  </si>
+  <si>
+    <t>26.98%</t>
+  </si>
+  <si>
+    <t>14.08</t>
+  </si>
+  <si>
+    <t>3.60%</t>
+  </si>
+  <si>
+    <t>9.73</t>
+  </si>
+  <si>
+    <t>26.63%</t>
+  </si>
+  <si>
+    <t>-11.49</t>
   </si>
   <si>
     <t>46.88%</t>
   </si>
   <si>
-    <t>-9.39</t>
-  </si>
-  <si>
-    <t>20.24%</t>
-  </si>
-  <si>
-    <t>-4.88</t>
+    <t>-8.74</t>
+  </si>
+  <si>
+    <t>20.25%</t>
+  </si>
+  <si>
+    <t>-4.74</t>
   </si>
   <si>
     <t>53.12%</t>
   </si>
   <si>
-    <t>9.39</t>
-  </si>
-  <si>
-    <t>Partição Total (PT)</t>
-  </si>
-  <si>
-    <t>12.45%</t>
-  </si>
-  <si>
-    <t>19.41%</t>
-  </si>
-  <si>
-    <t>-21.58</t>
-  </si>
-  <si>
-    <t>22.18%</t>
-  </si>
-  <si>
-    <t>34.41%</t>
-  </si>
-  <si>
-    <t>-16.50</t>
-  </si>
-  <si>
-    <t>α3 (riacho)</t>
-  </si>
-  <si>
-    <t>73.28%</t>
-  </si>
-  <si>
-    <t>84.12%</t>
-  </si>
-  <si>
-    <t>-5.60</t>
-  </si>
-  <si>
-    <t>9.73%</t>
-  </si>
-  <si>
-    <t>15.00%</t>
-  </si>
-  <si>
-    <t>-8.68</t>
-  </si>
-  <si>
-    <t>51.09%</t>
-  </si>
-  <si>
-    <t>49.72%</t>
-  </si>
-  <si>
-    <t>0.69</t>
-  </si>
-  <si>
-    <t>0.499</t>
-  </si>
-  <si>
-    <t>β3 (entre riachos)</t>
-  </si>
-  <si>
-    <t>26.72%</t>
-  </si>
-  <si>
-    <t>15.88%</t>
-  </si>
-  <si>
-    <t>5.60</t>
-  </si>
-  <si>
-    <t>23.72%</t>
-  </si>
-  <si>
-    <t>51.72%</t>
-  </si>
-  <si>
-    <t>-45.73</t>
-  </si>
-  <si>
-    <t>35.50%</t>
-  </si>
-  <si>
-    <t>69.45%</t>
-  </si>
-  <si>
-    <t>-35.41</t>
-  </si>
-  <si>
-    <t>83.75%</t>
-  </si>
-  <si>
-    <t>96.48%</t>
-  </si>
-  <si>
-    <t>-9.42</t>
-  </si>
-  <si>
-    <t>11.78%</t>
-  </si>
-  <si>
-    <t>17.73%</t>
-  </si>
-  <si>
-    <t>-7.46</t>
-  </si>
-  <si>
-    <t>48.25%</t>
-  </si>
-  <si>
-    <t>27.04%</t>
-  </si>
-  <si>
-    <t>13.64</t>
-  </si>
-  <si>
-    <t>16.25%</t>
-  </si>
-  <si>
-    <t>3.52%</t>
-  </si>
-  <si>
-    <t>9.42</t>
+    <t>8.74</t>
+  </si>
+  <si>
+    <t>44.01%</t>
+  </si>
+  <si>
+    <t>-20.57</t>
+  </si>
+  <si>
+    <t>61.70%</t>
+  </si>
+  <si>
+    <t>-13.60</t>
+  </si>
+  <si>
+    <t>17.69%</t>
+  </si>
+  <si>
+    <t>-3.16</t>
+  </si>
+  <si>
+    <t>38.30%</t>
+  </si>
+  <si>
+    <t>13.60</t>
+  </si>
+  <si>
+    <t>-15.13</t>
+  </si>
+  <si>
+    <t>38.50%</t>
+  </si>
+  <si>
+    <t>-10.40</t>
+  </si>
+  <si>
+    <t>16.03%</t>
+  </si>
+  <si>
+    <t>-4.40</t>
+  </si>
+  <si>
+    <t>61.50%</t>
+  </si>
+  <si>
+    <t>10.40</t>
+  </si>
+  <si>
+    <t>61.48%</t>
+  </si>
+  <si>
+    <t>-34.30</t>
+  </si>
+  <si>
+    <t>79.07%</t>
+  </si>
+  <si>
+    <t>-26.64</t>
+  </si>
+  <si>
+    <t>17.59%</t>
+  </si>
+  <si>
+    <t>-2.73</t>
+  </si>
+  <si>
+    <t>0.007*</t>
+  </si>
+  <si>
+    <t>20.93%</t>
+  </si>
+  <si>
+    <t>26.64</t>
   </si>
 </sst>
 </file>
@@ -650,807 +791,807 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>84</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G12" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="G14" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>111</v>
       </c>
       <c r="G15" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G18" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>91</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>94</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="E20" t="s">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="F20" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="E21" t="s">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
       <c r="G21" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="E22" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="F22" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="G22" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E23" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="F23" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="G23" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="E25" t="s">
-        <v>19</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>127</v>
       </c>
       <c r="G25" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E26" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="G26" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E27" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="F27" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G27" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B28" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>49</v>
       </c>
       <c r="G28" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>91</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>80</v>
+        <v>131</v>
       </c>
       <c r="F29" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="G29" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C30" t="s">
-        <v>14</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="G30" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E31" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="F31" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="G31" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="E32" t="s">
-        <v>19</v>
+        <v>137</v>
       </c>
       <c r="F32" t="s">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="G32" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C33" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="E33" t="s">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="F33" t="s">
-        <v>90</v>
+        <v>49</v>
       </c>
       <c r="G33" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B34" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C34" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D34" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E34" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="F34" t="s">
-        <v>93</v>
+        <v>140</v>
       </c>
       <c r="G34" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C35" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="D35" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E35" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
       <c r="F35" t="s">
-        <v>96</v>
+        <v>143</v>
       </c>
       <c r="G35" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1460,9 +1601,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A5EC255-ECD7-4415-A4B7-448500315BCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1489,787 +1630,788 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>100</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>101</v>
       </c>
       <c r="G9" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
+        <v>103</v>
       </c>
       <c r="G10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="F11" t="s">
-        <v>36</v>
+        <v>105</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="G12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>106</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="G13" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>108</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="G14" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>98</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E15" t="s">
-        <v>38</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>111</v>
       </c>
       <c r="G15" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
         <v>8</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E16" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="G18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" t="s">
         <v>18</v>
       </c>
-      <c r="D19" t="s">
-        <v>19</v>
-      </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>94</v>
       </c>
       <c r="D20" t="s">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E20" t="s">
-        <v>53</v>
+        <v>118</v>
       </c>
       <c r="F20" t="s">
-        <v>54</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="E21" t="s">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
       <c r="G21" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="E22" t="s">
-        <v>59</v>
+        <v>122</v>
       </c>
       <c r="F22" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="G22" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C23" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D23" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E23" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>63</v>
+        <v>11</v>
       </c>
       <c r="G23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="D24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E24" t="s">
-        <v>66</v>
+        <v>124</v>
       </c>
       <c r="F24" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="E25" t="s">
-        <v>19</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>127</v>
       </c>
       <c r="G25" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B26" t="s">
         <v>8</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E26" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="G26" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
         <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E27" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="F27" t="s">
-        <v>73</v>
+        <v>130</v>
       </c>
       <c r="G27" t="s">
-        <v>74</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B28" t="s">
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>9</v>
+        <v>91</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E29" t="s">
-        <v>80</v>
+        <v>131</v>
       </c>
       <c r="F29" t="s">
-        <v>81</v>
+        <v>132</v>
       </c>
       <c r="G29" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C30" t="s">
-        <v>14</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E30" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="G30" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="E31" t="s">
-        <v>86</v>
+        <v>135</v>
       </c>
       <c r="F31" t="s">
-        <v>87</v>
+        <v>136</v>
       </c>
       <c r="G31" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="D32" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="E32" t="s">
-        <v>19</v>
+        <v>137</v>
       </c>
       <c r="F32" t="s">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="G32" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C33" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="D33" t="s">
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="E33" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>90</v>
+        <v>11</v>
       </c>
       <c r="G33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B34" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C34" t="s">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="D34" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E34" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="F34" t="s">
-        <v>93</v>
+        <v>140</v>
       </c>
       <c r="G34" t="s">
-        <v>13</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="C35" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="D35" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E35" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
       <c r="F35" t="s">
-        <v>96</v>
+        <v>143</v>
       </c>
       <c r="G35" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>